<commit_message>
Atualizações 2024 e 18 RRAS
</commit_message>
<xml_diff>
--- a/f2_tabelas/tabela_idh_médio_por_rras.xlsx
+++ b/f2_tabelas/tabela_idh_médio_por_rras.xlsx
@@ -351,7 +351,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B20"/>
+  <dimension ref="A1:B19"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -369,191 +369,181 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>RRAS1</t>
+          <t>RRAS 1</t>
         </is>
       </c>
       <c r="B2">
-        <v>0.7943412642573806</v>
+        <v>0.7944121124527729</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>RRAS10</t>
+          <t>RRAS 2</t>
         </is>
       </c>
       <c r="B3">
-        <v>0.7681580137319703</v>
+        <v>0.7580313101043791</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>RRAS11</t>
+          <t>RRAS 3</t>
         </is>
       </c>
       <c r="B4">
-        <v>0.7644286710913342</v>
+        <v>0.7361030282723272</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>RRAS12</t>
+          <t>RRAS 4</t>
         </is>
       </c>
       <c r="B5">
-        <v>0.7699661836193139</v>
+        <v>0.7642237736164413</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>RRAS13</t>
+          <t>RRAS 5</t>
         </is>
       </c>
       <c r="B6">
-        <v>0.7682745311196907</v>
+        <v>0.7681016363053946</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>RRAS14</t>
+          <t>RRAS 6</t>
         </is>
       </c>
       <c r="B7">
-        <v>0.7739084357209086</v>
+        <v>0.805</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>RRAS15</t>
+          <t>RRAS 7</t>
         </is>
       </c>
       <c r="B8">
-        <v>0.7834546630046911</v>
+        <v>0.7617856857303096</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>RRAS16</t>
+          <t>RRAS 8</t>
         </is>
       </c>
       <c r="B9">
-        <v>0.7782573379739235</v>
+        <v>0.7574769932841702</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>RRAS17</t>
+          <t>RRAS 9</t>
         </is>
       </c>
       <c r="B10">
-        <v>0.781319874684563</v>
+        <v>0.7622949910726143</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>RRAS18</t>
+          <t>RRAS 10</t>
         </is>
       </c>
       <c r="B11">
-        <v>0.775532708823446</v>
+        <v>0.7679826641028091</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>RRAS19</t>
+          <t>RRAS 11</t>
         </is>
       </c>
       <c r="B12">
-        <v>0.7659403186838473</v>
+        <v>0.7644726722967612</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>RRAS2</t>
+          <t>RRAS 12</t>
         </is>
       </c>
       <c r="B13">
-        <v>0.7580370903022251</v>
+        <v>0.7686567262068865</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>RRAS3</t>
+          <t>RRAS 13</t>
         </is>
       </c>
       <c r="B14">
-        <v>0.7361663086391083</v>
+        <v>0.7683183228112802</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>RRAS4</t>
+          <t>RRAS 14</t>
         </is>
       </c>
       <c r="B15">
-        <v>0.7631194298172916</v>
+        <v>0.7738918443871573</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>RRAS5</t>
+          <t>RRAS 15</t>
         </is>
       </c>
       <c r="B16">
-        <v>0.7680397156956205</v>
+        <v>0.7834368421134841</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>RRAS6</t>
+          <t>RRAS 16</t>
         </is>
       </c>
       <c r="B17">
-        <v>0.805</v>
+        <v>0.7781862997381247</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>RRAS7</t>
+          <t>RRAS 17</t>
         </is>
       </c>
       <c r="B18">
-        <v>0.7618776272153588</v>
+        <v>0.7809834313551773</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>RRAS8</t>
+          <t>RRAS 18</t>
         </is>
       </c>
       <c r="B19">
-        <v>0.757446837506751</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>RRAS9</t>
-        </is>
-      </c>
-      <c r="B20">
-        <v>0.7623468749382887</v>
+        <v>0.775568279045705</v>
       </c>
     </row>
   </sheetData>

</xml_diff>